<commit_message>
Mirror LacksFurniture f748f59 for PR 54 device pass
</commit_message>
<xml_diff>
--- a/incoming/Lacks_Store_Data.xlsx
+++ b/incoming/Lacks_Store_Data.xlsx
@@ -6969,7 +6969,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"promotions":{"schemaVersion":1,"activeScenario":null,"allowedSourceHosts":["lacks.com"],"scenarios":{}},"financing":{"enabled":true,"experience":"payment-choice","offerVersion":"2026-07-30a","verifiedAt":"2026-07-31T16:43:00-05:00","maxAgeDays":7,"sourceUrl":"https://www.lacks.com/financing","applicationUrl":"https://www.lacks.com/credit-application","mexicoInfoUrl":"https://www.lacks.com/faq","mexicoApplicationUrl":{"url":"https://www.lacks.com/mexican-credit-application","verified":false,"note":"Published in Lacks' FAQ but returned 404 on 2026-07-30. Do not render as a link until it resolves; the Mexico card links to mexicoInfoUrl."},"savingsPassPolicy":"specialist_confirm","exactPromotionsEnabled":false,"esReviewStatus":"pending-native-legal-review","allowedSourceHosts":["lacks.com","www.lacks.com","synchrony.com","www.synchrony.com","mysynchrony.com"],"copy":{"eyebrow":{"en":"LACKS PAYMENT CHOICE","es":"OPCIONES DE PAGO LACKS"},"headline":{"en":"Better sleep. More ways to bring it home.","es":"Duerme mejor. Más opciones para llevarlo a casa."},"body":{"en":"Explore promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Options are subject to terms and approval.","es":"Explora financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. Las opciones están sujetas a términos y aprobación."},"cta":{"en":"Explore payment options","es":"Explorar opciones de pago"},"welcomeTagline":{"en":"Flexible ways to bring better sleep home.","es":"Formas flexibles de llevar mejor descanso a casa."},"welcomeSupport":{"en":"Explore payment options after finding your strongest mattress matches.","es":"Explora opciones de pago después de encontrar tus mejores opciones de colchón."},"resultsLead":{"en":"Your strongest mattress match may have more than one way to bring it home.","es":"Tu mejor opción de colchón puede tener más de una forma de llegar a casa."},"resultsAsk":{"en":"Plan the conversation","es":"Planear la conversación"},"fitFirst":{"en":"Your matches are based on sleep fit — never on payment method.","es":"Tus opciones se basan en tu descanso — nunca en la forma de pago."},"drawerTitle":{"en":"Ways to bring it home","es":"Formas de llevarlo a casa"},"drawerBody":{"en":"This recommendation is based on your sleep fit. When you're ready, Lacks offers more than one way to bring it home.","es":"Esta recomendación se basa en tu descanso. Cuando estés listo, Lacks ofrece más de una forma de llevarlo a casa."},"drawerMark":{"en":"Plan the conversation","es":"Planear la conversación"},"sleepSystemGuidance":{"en":"Build the sleep setup that fits you first. Your Lacks specialist can then review current payment options for the complete plan.","es":"Primero arma el sistema de sueño que te quede bien. Después, tu especialista de Lacks puede revisar las opciones de pago actuales para el plan completo."},"handoffHeadline":{"en":"Your Sleep Plan. Your Payment Choices.","es":"Tu Plan de Sueño. Tus Opciones de Pago."},"handoffPrivate":{"en":"Continue on your phone — scan to open Lacks' official financing page.","es":"Continúa desde tu teléfono — escanea para abrir la página oficial de financiamiento de Lacks."},"agendaPrompt":{"en":"As you review these together, mark any options the customer wants to discuss.","es":"Mientras revisan estas opciones juntos, marca las opciones de pago que el cliente quiera conversar."},"agendaMark":{"en":"Add to discussion","es":"Agregar a la conversación"},"agendaMarked":{"en":"Added to discussion","es":"Agregado a la conversación"},"agendaEmpty":{"en":"No options are marked yet.","es":"Todavía no hay opciones de pago marcadas."},"agendaConsequence":{"en":"Use this agenda to guide the conversation together. Nothing is submitted and no application is started.","es":"Usen esta agenda para guiar la conversación juntos. No se envía nada y no se inicia ninguna solicitud."},"agendaChange":{"en":"Change discussion agenda","es":"Cambiar agenda de conversación"},"agendaNotNow":{"en":"Not right now","es":"Ahora no"},"agendaDismissed":{"en":"No options marked for review right now.","es":"No hay opciones de pago marcadas para revisar por ahora."},"agendaDone":{"en":"Done","es":"Listo"},"interestNotNowAnnounce":{"en":"Not right now selected. You can change this choice.","es":"Se seleccionó 'Ahora no'. Puedes cambiar esta opción."},"interestClearedAnnounce":{"en":"Selection cleared. Choose again when you're ready.","es":"Se borró la selección. Elige de nuevo cuando quieras."},"staleNotice":{"en":"Current payment options are available from your Lacks specialist.","es":"Tu especialista de Lacks tiene las opciones de pago actuales."},"staleAnnouncement":{"en":"Exact rates and terms are not shown right now. Your Lacks specialist can confirm current payment options in store.","es":"Las tasas y los plazos exactos no se muestran en este momento. Tu especialista de Lacks puede confirmar las opciones de pago actuales en tienda."},"externalNotice":{"en":"Opens lacks.com — a separate site governed by its own terms and privacy policy.","es":"Abre lacks.com — un sitio aparte, regido por sus propios términos y política de privacidad."},"emailHeading":{"en":"Payment options","es":"Opciones de pago"},"emailBody":{"en":"You explored Lacks Payment Choice: promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Final pricing, eligibility, terms, and approval are confirmed by Lacks.","es":"Exploraste las Opciones de Pago Lacks: financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. El precio final, la elegibilidad, los términos y la aprobación los confirma Lacks."},"emailBodyAvailable":{"en":"Lacks Payment Choice offers more than one way to bring it home: promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Final pricing, eligibility, terms, and approval are confirmed by Lacks.","es":"Las Opciones de Pago Lacks ofrecen más de una forma de llevarlo a casa: financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. El precio final, la elegibilidad, los términos y la aprobación los confirma Lacks."},"disclosureFooter":{"en":"All payment options are subject to terms and approval. Advertised purchase minimums, rates, and terms are set by Lacks and its financing partners and may change or end at any time. Your Lacks specialist confirms current details in store.","es":"Todas las opciones de pago están sujetas a términos y aprobación. Los mínimos de compra, tasas y plazos anunciados los establecen Lacks y sus socios financieros y pueden cambiar o terminar en cualquier momento. Tu especialista de Lacks confirma los detalles vigentes en tienda."},"prequalNote":{"en":"See if you prequalify on Lacks' official financing page — prequalification is not approval.","es":"Consulta si precalificas en la página oficial de financiamiento de Lacks — precalificar no es una aprobación."}},"plans":[{"id":"synchrony-9-99-72","kind":"open-end-promotional-credit","provider":"Synchrony","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","apr":9.99,"termMonths":72,"minimumPurchase":500,"channel":"per-current-source","calculationMode":"published-fixed-factor","paymentCalculationEnabled":false,"headline":{"en":"9.99% APR for 72 months","es":"9.99% APR por 72 meses"},"detail":{"en":"On qualifying purchases of $500 or more with the Lacks Furniture Synchrony HOME Credit Card. Fixed monthly payments required. Interest is charged from the purchase date at the reduced APR. The advertised purchase minimum must be met on one receipt; discounts may reduce the purchase below it.","es":"En compras que califiquen de $500 o más con la tarjeta Lacks Furniture Synchrony HOME. Se requieren pagos mensuales fijos. Se cobra interés desde la fecha de compra a la tasa APR reducida. El mínimo de compra anunciado debe cumplirse en un solo recibo; los descuentos pueden reducir la compra por debajo del mínimo."},"disclosure":{"en":"Subject to credit approval. Regular account terms apply to non-promo purchases; for new accounts as of 07/31/2025 the purchase APR is 34.99%, penalty APR 39.99%, minimum interest charge $2. Lacks may alter or discontinue this offer at any time.","es":"Sujeto a aprobación de crédito. Los términos regulares de la cuenta aplican a compras fuera de promoción; para cuentas nuevas al 07/31/2025 la tasa APR de compra es 34.99%, la APR de penalización 39.99% y el cargo mínimo por interés $2. Lacks puede modificar o descontinuar esta oferta en cualquier momento."}},{"id":"synchrony-0-48","kind":"open-end-promotional-credit","provider":"Synchrony","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","apr":0,"termMonths":48,"minimumPurchase":4200,"channel":"in-store","calculationMode":"not-published","paymentCalculationEnabled":false,"headline":{"en":"0% APR for 48 months","es":"0% APR por 48 meses"},"detail":{"en":"On qualifying in-store purchases of $4,200 or more with the Lacks Furniture Synchrony HOME Credit Card. Equal monthly payments required. A minimum purchase and a down payment, plus tax and delivery fee, are required. The advertised purchase minimum must be met on one receipt; discounts may reduce the purchase below it.","es":"En compras en tienda que califiquen de $4,200 o más con la tarjeta Lacks Furniture Synchrony HOME. Se requieren pagos mensuales iguales. Se requiere una compra mínima y un enganche, más impuestos y cargo de entrega. El mínimo de compra anunciado debe cumplirse en un solo recibo; los descuentos pueden reducir la compra por debajo del mínimo."},"disclosure":{"en":"Subject to credit approval. No interest is charged on the promotional purchase. Regular account terms apply to non-promo purchases; for new accounts as of 07/31/2025 the purchase APR is 34.99%, penalty APR 39.99%, minimum interest charge $2.","es":"Sujeto a aprobación de crédito. No se cobra interés en la compra promocional. Los términos regulares de la cuenta aplican a compras fuera de promoción; para cuentas nuevas al 07/31/2025 la tasa APR de compra es 34.99%, la APR de penalización 39.99% y el cargo mínimo por interés $2."}},{"id":"lacks-in-house","kind":"closed-end-installment","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Lacks In-House Credit","es":"Crédito Interno de Lacks"},"detail":{"en":"Installment contracts may be available from 6–36 months for qualifying customers, with in-house approvals by Lacks' own credit team. Purchases may also qualify for promotional pricing. Subject to Lacks approval and applicable offer terms.","es":"Para clientes que califiquen, puede haber contratos a plazos de 6 a 36 meses, con aprobación interna del propio equipo de crédito de Lacks. Las compras también pueden calificar para precios promocionales. Sujeto a la aprobación de Lacks y a los términos de la oferta aplicable."},"disclosure":{"en":"Availability, terms, and promotional pricing are confirmed by Lacks in store.","es":"La disponibilidad, los términos y los precios promocionales los confirma Lacks en tienda."}},{"id":"lease-to-own","kind":"lease-to-own","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Lease-to-own","es":"Arrendamiento con opción a compra"},"detail":{"en":"Lease-to-own is available. Program details, costs, eligibility, and ownership terms are confirmed in store.","es":"El arrendamiento con opción a compra está disponible. Los detalles del programa, costos, elegibilidad y términos de propiedad se confirman en tienda."}},{"id":"build-my-credit","kind":"credit-builder","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Build My Credit","es":"Build My Credit"},"detail":{"en":"An available path for customers with little or no credit history. Program details are confirmed in store.","es":"Una opción disponible para clientes con poco o ningún historial de crédito. Los detalles del programa se confirman en tienda."}},{"id":"mexico-in-house","kind":"closed-end-installment","provider":"Lacks","presentationScenario":"mexico-delivery","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/faq","apr":24,"termMonths":24,"paymentCalculationEnabled":false,"headline":{"en":"Purchasing for delivery to Mexico?","es":"¿Compras para entrega en México?"},"detail":{"en":"An optional program for customers purchasing for delivery to Mexico: Lacks in-house credit for up to 24 months with a maximum contract APR of 24% (which may vary). Requirements currently include two official IDs, three personal references, and income verification.","es":"Un programa opcional para clientes que compran para entrega en México: crédito interno de Lacks hasta por 24 meses con un interés máximo del contrato de 24% APR (mismo que puede variar). Los requisitos actuales incluyen dos identificaciones oficiales, 3 referencias personales y verificación de ingresos."},"representativeExample":{"en":"Lacks' published example: $999 financed for 24 months at 24% APR equals 24 monthly payments of $52.82.","es":"Ejemplo publicado por Lacks: $999 financiados durante 24 meses con 24% APR tendrán 24 pagos mensuales de $52.82."},"disclosure":{"en":"For purchases intended for delivery to Mexico, ask a Lacks specialist to confirm current details and requirements.","es":"Para compras destinadas a entrega en México, consulta con un especialista de Lacks para confirmar los detalles y requisitos actuales."}}]}}</t>
+          <t>{"promotions":{"schemaVersion":1,"activeScenario":null,"allowedSourceHosts":["lacks.com"],"scenarios":{}},"financing":{"enabled":true,"experience":"payment-choice","offerVersion":"2026-07-30a","verifiedAt":"2026-07-31T16:43:00-05:00","maxAgeDays":7,"sourceUrl":"https://www.lacks.com/financing","applicationUrl":"https://www.lacks.com/credit-application","mexicoInfoUrl":"https://www.lacks.com/faq","mexicoApplicationUrl":{"url":"https://www.lacks.com/mexican-credit-application","verified":false,"note":"Published in Lacks' FAQ but returned 404 on 2026-07-30. Do not render as a link until it resolves; the Mexico card links to mexicoInfoUrl."},"savingsPassPolicy":"specialist_confirm","exactPromotionsEnabled":false,"esReviewStatus":"pending-native-legal-review","surfaces":{"drawer":false,"sleepSystem":false},"allowedSourceHosts":["lacks.com","www.lacks.com","synchrony.com","www.synchrony.com","mysynchrony.com"],"copy":{"eyebrow":{"en":"LACKS PAYMENT CHOICE","es":"OPCIONES DE PAGO LACKS"},"headline":{"en":"Better sleep. More ways to bring it home.","es":"Duerme mejor. Más opciones para llevarlo a casa."},"body":{"en":"Explore promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Options are subject to terms and approval.","es":"Explora financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. Las opciones están sujetas a términos y aprobación."},"cta":{"en":"Explore payment options","es":"Explorar opciones de pago"},"welcomeTagline":{"en":"Flexible ways to bring better sleep home.","es":"Formas flexibles de llevar mejor descanso a casa."},"welcomeSupport":{"en":"Explore payment options after finding your strongest mattress matches.","es":"Explora opciones de pago después de encontrar tus mejores opciones de colchón."},"resultsLead":{"en":"Your strongest mattress match may have more than one way to bring it home.","es":"Tu mejor opción de colchón puede tener más de una forma de llegar a casa."},"fitFirst":{"en":"Your matches are based on sleep fit — never on payment method.","es":"Tus opciones se basan en tu descanso — nunca en la forma de pago."},"drawerTitle":{"en":"Ways to bring it home","es":"Formas de llevarlo a casa"},"drawerBody":{"en":"This recommendation is based on your sleep fit. When you're ready, Lacks offers more than one way to bring it home.","es":"Esta recomendación se basa en tu descanso. Cuando estés listo, Lacks ofrece más de una forma de llevarlo a casa."},"sleepSystemGuidance":{"en":"Build the sleep setup that fits you first. Your Lacks specialist can then review current payment options for the complete plan.","es":"Primero arma el sistema de sueño que te quede bien. Después, tu especialista de Lacks puede revisar las opciones de pago actuales para el plan completo."},"handoffHeadline":{"en":"Your Sleep Plan. Your Payment Choices.","es":"Tu Plan de Sueño. Tus Opciones de Pago."},"handoffPrivate":{"en":"Continue on your phone — scan to open Lacks' official financing page.","es":"Continúa desde tu teléfono — escanea para abrir la página oficial de financiamiento de Lacks."},"paymentPreferenceLabel":{"en":"Payment preference","es":"Preferencia de pago"},"preferenceNone":{"en":"Not selected","es":"Sin seleccionar"},"optionsExploredLabel":{"en":"Options explored","es":"Opciones exploradas"},"reviewOption":{"en":"Review this option","es":"Revisar esta opción"},"hideDetails":{"en":"Hide details","es":"Ocultar detalles"},"considerOption":{"en":"Consider this option","es":"Considerar esta opción"},"currentlyConsidering":{"en":"Currently considering ✓","es":"En consideración ✓"},"clearPreference":{"en":"Clear preference","es":"Quitar preferencia"},"preferenceNotNow":{"en":"Not right now","es":"Ahora no"},"exploreConsequence":{"en":"Explore options together. Nothing is submitted and no application is started.","es":"Exploren las opciones juntos. No se envía nada y no se inicia ninguna solicitud."},"sheetDone":{"en":"Done","es":"Listo"},"preferenceNotNowAnnounce":{"en":"Not right now selected. You can change this choice.","es":"Se seleccionó 'Ahora no'. Puedes cambiar esta opción."},"preferenceClearedAnnounce":{"en":"Selection cleared. Choose again when you're ready.","es":"Se borró la selección. Elige de nuevo cuando quieras."},"staleNotice":{"en":"Current payment options are available from your Lacks specialist.","es":"Tu especialista de Lacks tiene las opciones de pago actuales."},"staleAnnouncement":{"en":"Exact rates and terms are not shown right now. Your Lacks specialist can confirm current payment options in store.","es":"Las tasas y los plazos exactos no se muestran en este momento. Tu especialista de Lacks puede confirmar las opciones de pago actuales en tienda."},"externalNotice":{"en":"Opens lacks.com — a separate site governed by its own terms and privacy policy.","es":"Abre lacks.com — un sitio aparte, regido por sus propios términos y política de privacidad."},"emailHeading":{"en":"Payment options","es":"Opciones de pago"},"emailBodyAvailable":{"en":"Lacks Payment Choice offers more than one way to bring it home: promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Final pricing, eligibility, terms, and approval are confirmed by Lacks.","es":"Las Opciones de Pago Lacks ofrecen más de una forma de llevarlo a casa: financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. El precio final, la elegibilidad, los términos y la aprobación los confirma Lacks."},"disclosureFooter":{"en":"All payment options are subject to terms and approval. Advertised purchase minimums, rates, and terms are set by Lacks and its financing partners and may change or end at any time. Your Lacks specialist confirms current details in store.","es":"Todas las opciones de pago están sujetas a términos y aprobación. Los mínimos de compra, tasas y plazos anunciados los establecen Lacks y sus socios financieros y pueden cambiar o terminar en cualquier momento. Tu especialista de Lacks confirma los detalles vigentes en tienda."},"prequalNote":{"en":"See if you prequalify on Lacks' official financing page — prequalification is not approval.","es":"Consulta si precalificas en la página oficial de financiamiento de Lacks — precalificar no es una aprobación."}},"plans":[{"id":"synchrony-9-99-72","kind":"open-end-promotional-credit","provider":"Synchrony","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","apr":9.99,"termMonths":72,"minimumPurchase":500,"channel":"per-current-source","calculationMode":"published-fixed-factor","paymentCalculationEnabled":false,"headline":{"en":"9.99% APR for 72 months","es":"9.99% APR por 72 meses"},"detail":{"en":"On qualifying purchases of $500 or more with the Lacks Furniture Synchrony HOME Credit Card. Fixed monthly payments required. Interest is charged from the purchase date at the reduced APR. The advertised purchase minimum must be met on one receipt; discounts may reduce the purchase below it.","es":"En compras que califiquen de $500 o más con la tarjeta Lacks Furniture Synchrony HOME. Se requieren pagos mensuales fijos. Se cobra interés desde la fecha de compra a la tasa APR reducida. El mínimo de compra anunciado debe cumplirse en un solo recibo; los descuentos pueden reducir la compra por debajo del mínimo."},"disclosure":{"en":"Subject to credit approval. Regular account terms apply to non-promo purchases; for new accounts as of 07/31/2025 the purchase APR is 34.99%, penalty APR 39.99%, minimum interest charge $2. Lacks may alter or discontinue this offer at any time.","es":"Sujeto a aprobación de crédito. Los términos regulares de la cuenta aplican a compras fuera de promoción; para cuentas nuevas al 07/31/2025 la tasa APR de compra es 34.99%, la APR de penalización 39.99% y el cargo mínimo por interés $2. Lacks puede modificar o descontinuar esta oferta en cualquier momento."}},{"id":"synchrony-0-48","kind":"open-end-promotional-credit","provider":"Synchrony","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","apr":0,"termMonths":48,"minimumPurchase":4200,"channel":"in-store","calculationMode":"not-published","paymentCalculationEnabled":false,"headline":{"en":"0% APR for 48 months","es":"0% APR por 48 meses"},"detail":{"en":"On qualifying in-store purchases of $4,200 or more with the Lacks Furniture Synchrony HOME Credit Card. Equal monthly payments required. A minimum purchase and a down payment, plus tax and delivery fee, are required. The advertised purchase minimum must be met on one receipt; discounts may reduce the purchase below it.","es":"En compras en tienda que califiquen de $4,200 o más con la tarjeta Lacks Furniture Synchrony HOME. Se requieren pagos mensuales iguales. Se requiere una compra mínima y un enganche, más impuestos y cargo de entrega. El mínimo de compra anunciado debe cumplirse en un solo recibo; los descuentos pueden reducir la compra por debajo del mínimo."},"disclosure":{"en":"Subject to credit approval. No interest is charged on the promotional purchase. Regular account terms apply to non-promo purchases; for new accounts as of 07/31/2025 the purchase APR is 34.99%, penalty APR 39.99%, minimum interest charge $2.","es":"Sujeto a aprobación de crédito. No se cobra interés en la compra promocional. Los términos regulares de la cuenta aplican a compras fuera de promoción; para cuentas nuevas al 07/31/2025 la tasa APR de compra es 34.99%, la APR de penalización 39.99% y el cargo mínimo por interés $2."}},{"id":"lacks-in-house","kind":"closed-end-installment","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Lacks In-House Credit","es":"Crédito Interno de Lacks"},"detail":{"en":"Installment contracts may be available from 6–36 months for qualifying customers, with in-house approvals by Lacks' own credit team. Purchases may also qualify for promotional pricing. Subject to Lacks approval and applicable offer terms.","es":"Para clientes que califiquen, puede haber contratos a plazos de 6 a 36 meses, con aprobación interna del propio equipo de crédito de Lacks. Las compras también pueden calificar para precios promocionales. Sujeto a la aprobación de Lacks y a los términos de la oferta aplicable."},"disclosure":{"en":"Availability, terms, and promotional pricing are confirmed by Lacks in store.","es":"La disponibilidad, los términos y los precios promocionales los confirma Lacks en tienda."}},{"id":"lease-to-own","kind":"lease-to-own","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Lease-to-own","es":"Arrendamiento con opción a compra"},"detail":{"en":"Lease-to-own is available. Program details, costs, eligibility, and ownership terms are confirmed in store.","es":"El arrendamiento con opción a compra está disponible. Los detalles del programa, costos, elegibilidad y términos de propiedad se confirman en tienda."}},{"id":"build-my-credit","kind":"credit-builder","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Build My Credit","es":"Build My Credit"},"detail":{"en":"An available path for customers with little or no credit history. Program details are confirmed in store.","es":"Una opción disponible para clientes con poco o ningún historial de crédito. Los detalles del programa se confirman en tienda."}},{"id":"mexico-in-house","kind":"closed-end-installment","provider":"Lacks","presentationScenario":"mexico-delivery","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/faq","apr":24,"termMonths":24,"paymentCalculationEnabled":false,"headline":{"en":"Purchasing for delivery to Mexico?","es":"¿Compras para entrega en México?"},"detail":{"en":"An optional program for customers purchasing for delivery to Mexico: Lacks in-house credit for up to 24 months with a maximum contract APR of 24% (which may vary). Requirements currently include two official IDs, three personal references, and income verification.","es":"Un programa opcional para clientes que compran para entrega en México: crédito interno de Lacks hasta por 24 meses con un interés máximo del contrato de 24% APR (mismo que puede variar). Los requisitos actuales incluyen dos identificaciones oficiales, 3 referencias personales y verificación de ingresos."},"representativeExample":{"en":"Lacks' published example: $999 financed for 24 months at 24% APR equals 24 monthly payments of $52.82.","es":"Ejemplo publicado por Lacks: $999 financiados durante 24 meses con 24% APR tendrán 24 pagos mensuales de $52.82."},"disclosure":{"en":"For purchases intended for delivery to Mexico, ask a Lacks specialist to confirm current details and requirements.","es":"Para compras destinadas a entrega en México, consulta con un especialista de Lacks para confirmar los detalles y requisitos actuales."}}]}}</t>
         </is>
       </c>
     </row>
@@ -6997,7 +6997,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"quiz":{"questions":[{"id":"trigger","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What can we help you with today?","es":"¿En qué te podemos ayudar hoy?"},"helpText":{"en":"No pressure — this just helps your specialist focus on what matters to you.","es":"Sin presión — esto ayuda a tu especialista a enfocarse en lo que te importa."},"type":"single","options":[{"id":"pain","label":{"en":"Back or Body Pain","es":"Dolor de Espalda o Cuerpo"},"icon":"spine","sublabel":{"en":"Current mattress is hurting me","es":"Mi colchón actual me lastima"},"scores":{}},{"id":"worn_out","label":{"en":"Old Mattress","es":"Colchón Viejo"},"icon":"sagging","sublabel":{"en":"Time for an upgrade","es":"Es hora de un cambio"},"scores":{}},{"id":"moving","label":{"en":"Moving or New Space","es":"Mudanza o Espacio Nuevo"},"icon":"family","sublabel":{"en":"New home, new bed","es":"Casa nueva, cama nueva"},"scores":{}},{"id":"upgrade","label":{"en":"Just Upgrading","es":"Mejorando"},"icon":"cloud","sublabel":{"en":"Ready for something better","es":"Listo para algo mejor"},"scores":{}},{"id":"browsing","label":{"en":"Just Browsing","es":"Solo Explorando"},"icon":"smile","sublabel":{"en":"Getting ideas, no rush","es":"Sin prisa, juntando ideas"},"scores":{}}]},{"id":"mattress_size","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What size mattress are you looking for?","es":"¿Qué tamaño de colchón buscas?"},"helpText":{"en":"So every mattress we show actually fits your space.","es":"Nos aseguraremos de que las recomendaciones se ajusten a tu espacio"},"type":"single","options":[{"id":"twin","label":{"en":"Twin","es":"Twin"},"icon":"solo","sublabel":{"en":"Kids or tight spaces","es":"Niños o espacios pequeños"},"scores":{}},{"id":"twin_xl","label":{"en":"Twin XL","es":"Twin XL"},"icon":"solo","sublabel":{"en":"Extra length, single sleeper","es":"Largo extra, una persona"},"scores":{}},{"id":"full","label":{"en":"Full","es":"Full"},"icon":"solo","sublabel":{"en":"Solo or cozy pair","es":"Solo o pareja cómoda"},"scores":{}},{"id":"queen","label":{"en":"Queen","es":"Queen"},"icon":"partner","sublabel":{"en":"Most popular size","es":"El tamaño más popular"},"scores":{}},{"id":"king","label":{"en":"King","es":"King"},"icon":"family","sublabel":{"en":"Maximum space","es":"Espacio máximo"},"scores":{}},{"id":"cal_king","label":{"en":"Cal King","es":"Cal King"},"icon":"family","sublabel":{"en":"Extra length","es":"Largo extra"},"scores":{}}]},{"id":"partner_sleep","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Who's sharing the bed with you?","es":"¿Quién comparte la cama contigo?"},"helpText":{"en":"Who shares your bed shapes which features matter most.","es":"Esto determina qué características importan más"},"type":"single","options":[{"id":"solo","label":{"en":"Solo Sleeper","es":"Duermo Solo"},"icon":"solo","sublabel":{"en":"Just me","es":"Solo yo"},"scores":{}},{"id":"partner","label":{"en":"With a Partner","es":"Con Pareja"},"icon":"partner","sublabel":{"en":"Sharing the bed","es":"Compartimos la cama"},"scores":{"motionIsolation":2}},{"id":"family","label":{"en":"Family Bed","es":"Cama Familiar"},"icon":"family","sublabel":{"en":"Kids, pets, or both","es":"Niños, mascotas, o ambos"},"scores":{"durability":2,"motionIsolation":1}}]},{"id":"partner_disturbance","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Does your partner's movement wake you up?","es":"¿El movimiento de tu pareja te despierta?"},"helpText":{"en":"Motion isolation is one of the first upgrades you'll feel.","es":"El aislamiento de movimiento es una de las mayores mejoras en un colchón nuevo"},"type":"single","skipIf":{"question":"partner_sleep","answer":"solo"},"options":[{"id":"yes_often","label":{"en":"Yes, Often","es":"Sí, Seguido"},"icon":"motion","sublabel":{"en":"Every movement wakes me","es":"Cada movimiento me despierta"},"scores":{"motionIsolation":4,"hybrid":3,"memory":2}},{"id":"sometimes","label":{"en":"Sometimes","es":"A Veces"},"icon":"combo","sublabel":{"en":"Bigger movements bother me","es":"Los movimientos grandes me molestan"},"scores":{"motionIsolation":3,"hybrid":2}},{"id":"rarely","label":{"en":"Rarely","es":"Rara Vez"},"icon":"check","sublabel":{"en":"Light sleeper but mostly fine","es":"Sueño ligero pero generalmente bien"},"scores":{"motionIsolation":1}},{"id":"not_applicable","label":{"en":"Doesn't Apply","es":"No Aplica"},"icon":"solo","sublabel":{"en":"I sleep alone","es":"Duermo solo"},"scores":{}}]},{"id":"sleep_position","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"How do you usually sleep?","es":"¿Cómo duermes normalmente?"},"helpText":{"en":"Your sleep position is the biggest clue to the support you need.","es":"Piensa en cómo terminas naturalmente"},"type":"single","options":[{"id":"side","label":{"en":"Side Sleeper","es":"De Lado"},"icon":"side","sublabel":{"en":"Curled up","es":"Acurrucado"},"scores":{"plush":2,"pressureRelief":2,"soft":1}},{"id":"back","label":{"en":"Back Sleeper","es":"Boca Arriba"},"icon":"back","sublabel":{"en":"Flat on back","es":"Acostado de espalda"},"scores":{"support":2,"medium":2,"zoned":1}},{"id":"stomach","label":{"en":"Stomach Sleeper","es":"Boca Abajo"},"icon":"stomach","sublabel":{"en":"Face down","es":"Boca abajo"},"scores":{"firm":2,"support":1}},{"id":"combo","label":{"en":"Combination","es":"Combinación"},"icon":"combo","sublabel":{"en":"Move around","es":"Me muevo mucho"},"scores":{"medium":2,"responsive":2}},{"id":"no_idea","label":{"en":"Not Sure","es":"No Estoy Seguro"},"icon":"question","sublabel":{"en":"I wake up in weird positions","es":"Me despierto en posiciones raras"},"scores":{"medium":2,"responsive":2}}]},{"id":"body_type","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"What weight range should this mattress support?","es":"¿Qué rango de peso debe soportar este colchón?"},"helpText":{"en":"This helps us account for cushioning, support, and durability.","es":"Esto nos ayuda a considerar la amortiguación, el soporte y la durabilidad."},"type":"single","options":[{"id":"petite","label":{"en":"Under 130 lbs","es":"Menos de 130 lbs"},"icon":"cloud","sublabel":{"en":"Light support","es":"Soporte ligero"},"scores":{"plush":2,"soft":1}},{"id":"average","label":{"en":"130 to 200 lbs","es":"130 a 200 lbs"},"icon":"weight","sublabel":{"en":"Standard support","es":"Soporte estándar"},"scores":{"medium":2}},{"id":"athletic","label":{"en":"200 to 230 lbs","es":"200 a 230 lbs"},"icon":"support","sublabel":{"en":"Medium-firm support","es":"Soporte medio-firme"},"scores":{"support":2,"medium":1,"responsive":1}},{"id":"plus","label":{"en":"Over 230 lbs","es":"Más de 230 lbs"},"icon":"support","sublabel":{"en":"Maximum support","es":"Soporte máximo"},"scores":{"firm":2,"support":3,"hybrid":2,"durability":2}},{"id":"different","label":{"en":"Different weight ranges","es":"Rangos de peso diferentes"},"icon":"partner","sublabel":{"en":"Sleepers fall into different ranges","es":"Los durmientes están en rangos diferentes"},"scores":{"medium":2,"support":1,"motionIsolation":2},"hideIf":{"question":"partner_sleep","answer":"solo"}}],"copyVariants":[{"when":{"question":"partner_sleep","answerIn":["partner","family"]},"question":{"en":"What weight range should we match for the sleeper who needs more support?","es":"¿Para qué rango de peso debemos ajustar, según quien necesite más soporte?"},"helpText":{"en":"If you fall into different ranges, choose “Different weight ranges.”","es":"Si están en rangos diferentes, elige “Rangos de peso diferentes”."}}]},{"id":"temperature","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"How do you sleep temperature-wise?","es":"¿Cómo duermes en cuanto a temperatura?"},"helpText":{"en":"Sleeping hot or cold is an easy fix with the right materials.","es":"La regulación de temperatura es clave para un sueño profundo"},"type":"single","options":[{"id":"hot","label":{"en":"I Sleep Hot","es":"Duermo con Calor"},"icon":"flame","sublabel":{"en":"Night sweats, kick off covers","es":"Sudores nocturnos, quito las cobijas"},"scores":{"cooling":3,"hybrid":2}},{"id":"comfortable","label":{"en":"I'm Comfortable","es":"Estoy Cómodo"},"icon":"smile","sublabel":{"en":"No temperature issues","es":"Sin problemas de temperatura"},"scores":{}},{"id":"cold","label":{"en":"I Sleep Cold","es":"Duermo con Frío"},"icon":"snowflake","sublabel":{"en":"Need blankets to warm up","es":"Necesito cobijas para calentarme"},"scores":{"memory":1,"plush":1}},{"id":"opposite","label":{"en":"We're Opposite","es":"Somos Opuestos"},"icon":"hotcold","sublabel":{"en":"One hot, one cold","es":"Uno con calor, otro con frío"},"scores":{"cooling":2,"hybrid":1},"hideIf":{"question":"partner_sleep","answer":"solo"}}]},{"id":"firmness","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"What firmness level do you prefer?","es":"¿Qué nivel de firmeza prefieres?"},"helpText":{"en":"No wrong answer here, just slide to what feels best.","es":"Desliza a tu comodidad ideal"},"type":"slider","min":1,"max":10,"defaultValue":5,"labels":[{"en":"Soft — Sink right in","es":"Suave — Hundirse"},{"en":"Medium","es":"Medio"},{"en":"Firm — Solid support","es":"Firme — Soporte sólido"}]},{"id":"sleep_issues","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Any issues with your current mattress?","es":"¿Algún problema con tu colchón actual?"},"helpText":{"en":"Tap anything you've noticed. Each one points us toward a fix.","es":"Toca las que apliquen"},"type":"multiple","options":[{"id":"back_pain","label":{"en":"Back Pain","es":"Dolor de Espalda"},"icon":"spine","sublabel":{"en":"Lower or upper back","es":"Espalda baja o alta"},"scores":{"support":3,"zoned":2,"firm":1}},{"id":"hip_pain","label":{"en":"Hip or Shoulder Pain","es":"Dolor de Cadera u Hombro"},"icon":"pressure","sublabel":{"en":"Pressure points","es":"Puntos de presión"},"scores":{"pressureRelief":3,"plush":2}},{"id":"hot","label":{"en":"Sleeping Too Hot","es":"Mucho Calor al Dormir"},"icon":"flame","sublabel":{"en":"Night sweats, overheating","es":"Sudores nocturnos, sobrecalentamiento"},"scores":{"cooling":3,"hybrid":2}},{"id":"tossing","label":{"en":"Tossing &amp; Turning","es":"Dando Vueltas"},"icon":"combo","sublabel":{"en":"Can't get comfortable","es":"No encuentro comodidad"},"scores":{"comfort":2,"medium":1}},{"id":"stiff","label":{"en":"Waking Up Stiff or Sore","es":"Despertar Rígido o Adolorido"},"icon":"stiff","sublabel":{"en":"Morning aches","es":"Dolores matutinos"},"scores":{"pressureRelief":2,"comfort":2}},{"id":"sagging","label":{"en":"Mattress Sagging","es":"Colchón Hundido"},"icon":"sagging","sublabel":{"en":"Dips or indentations","es":"Hundimientos"},"scores":{"durability":2,"quality":2}},{"id":"too_soft","label":{"en":"Mattress Too Soft","es":"Colchón Muy Suave"},"icon":"couch","sublabel":{"en":"Sinking in too much","es":"Me hundo demasiado"},"scores":{"firm":3,"support":2}},{"id":"none","label":{"en":"No Major Issues","es":"Sin Problemas Grandes"},"icon":"check","sublabel":{"en":"Just time for an upgrade","es":"Solo es hora de un cambio"},"scores":{"comfort":1,"quality":1,"durable":1}}]},{"id":"health_conditions","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Anything else going on that affects your sleep?","es":"¿Algo más que afecte tu sueño?"},"helpText":{"en":"Tap any that apply. A few of these change what we'd suggest.","es":"Toca las que apliquen"},"type":"multiple","options":[{"id":"nerve_pain","label":{"en":"Nerve Pain or Tingling","es":"Dolor Nervioso u Hormigueo"},"icon":"lightning","sublabel":{"en":"Shooting pain, numbness","es":"Dolor punzante, entumecimiento"},"scores":{"support":3,"firm":2,"zoned":2}},{"id":"allergies","label":{"en":"Allergies","es":"Alergias"},"icon":"sneeze","sublabel":{"en":"Dust, sneezing, stuffy","es":"Polvo, estornudos, congestión"},"scores":{"hypoallergenic":3}},{"id":"snoring","label":{"en":"Snoring or Sleep Apnea","es":"Ronquidos o Apnea del Sueño"},"icon":"snore","sublabel":{"en":"You or your partner","es":"Tú o tu pareja"},"scores":{"adjustable":3}},{"id":"reflux","label":{"en":"Acid Reflux / Heartburn","es":"Reflujo Ácido / Acidez"},"icon":"flame","sublabel":{"en":"Burns when lying down","es":"Arde al acostarse"},"scores":{"adjustable":3}},{"id":"extra_support","label":{"en":"Need Extra Support","es":"Necesito Soporte Extra"},"icon":"weight","sublabel":{"en":"Larger build or heavier weight","es":"Complexión grande o peso mayor"},"scores":{"support":3,"firm":2,"durable":3}},{"id":"getting_older","label":{"en":"Changing Needs","es":"Necesidades Cambiantes"},"icon":"aging","sublabel":{"en":"Looking for gentler support","es":"Buscando soporte más suave"},"scores":{"support":2,"comfort":2,"pressureRelief":1}},{"id":"none","label":{"en":"None of These","es":"Ninguno de Estos"},"icon":"check","sublabel":{"en":"I'm good","es":"Estoy bien"},"scores":{}}]}]}}</t>
+          <t>{"quiz":{"questions":[{"id":"trigger","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What can we help you with today?","es":"¿En qué te podemos ayudar hoy?"},"helpText":{"en":"This doesn't change your sleep-fit ranking. It helps your specialist focus on what matters to you.","es":"Esto no cambia el orden de tus opciones. Ayuda a tu especialista a enfocarse en lo que te importa."},"type":"single","options":[{"id":"pain","label":{"en":"Back or Body Pain","es":"Dolor de Espalda o Cuerpo"},"icon":"spine","sublabel":{"en":"Current mattress is hurting me","es":"Mi colchón actual me lastima"},"scores":{}},{"id":"worn_out","label":{"en":"Old Mattress","es":"Colchón Viejo"},"icon":"sagging","sublabel":{"en":"Time for an upgrade","es":"Es hora de un cambio"},"scores":{}},{"id":"moving","label":{"en":"Moving or New Space","es":"Mudanza o Espacio Nuevo"},"icon":"family","sublabel":{"en":"New home, new bed","es":"Casa nueva, cama nueva"},"scores":{}},{"id":"upgrade","label":{"en":"Just Upgrading","es":"Mejorando"},"icon":"cloud","sublabel":{"en":"Ready for something better","es":"Listo para algo mejor"},"scores":{}},{"id":"browsing","label":{"en":"Just Browsing","es":"Solo Explorando"},"icon":"smile","sublabel":{"en":"Getting ideas, no rush","es":"Sin prisa, juntando ideas"},"scores":{}}]},{"id":"mattress_size","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What size mattress are you looking for?","es":"¿Qué tamaño de colchón buscas?"},"helpText":{"en":"We carry your selected size into the consultation. Your sleep-fit ranking is based on your comfort and support answers.","es":"Tomamos en cuenta el tamaño que elijas en la consulta. El orden de tus opciones se basa en tus respuestas sobre comodidad y soporte."},"type":"single","options":[{"id":"twin","label":{"en":"Twin","es":"Twin"},"icon":"solo","sublabel":{"en":"Kids or tight spaces","es":"Niños o espacios pequeños"},"scores":{}},{"id":"twin_xl","label":{"en":"Twin XL","es":"Twin XL"},"icon":"solo","sublabel":{"en":"Extra length, single sleeper","es":"Largo extra, una persona"},"scores":{}},{"id":"full","label":{"en":"Full","es":"Full"},"icon":"solo","sublabel":{"en":"Solo or cozy pair","es":"Solo o pareja cómoda"},"scores":{}},{"id":"queen","label":{"en":"Queen","es":"Queen"},"icon":"partner","sublabel":{"en":"Most popular size","es":"El tamaño más popular"},"scores":{}},{"id":"king","label":{"en":"King","es":"King"},"icon":"family","sublabel":{"en":"Maximum space","es":"Espacio máximo"},"scores":{}},{"id":"cal_king","label":{"en":"Cal King","es":"Cal King"},"icon":"family","sublabel":{"en":"Extra length","es":"Largo extra"},"scores":{}}]},{"id":"partner_sleep","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Who's sharing the bed with you?","es":"¿Quién comparte la cama contigo?"},"helpText":{"en":"This shapes the questions that follow and what we suggest testing together.","es":"Esto define las preguntas que siguen y lo que sugerimos probar juntos."},"type":"single","options":[{"id":"solo","label":{"en":"Solo Sleeper","es":"Duermo Solo"},"icon":"solo","sublabel":{"en":"Just me","es":"Solo yo"},"scores":{}},{"id":"partner","label":{"en":"With a Partner","es":"Con Pareja"},"icon":"partner","sublabel":{"en":"Sharing the bed","es":"Compartimos la cama"},"scores":{"motionIsolation":2}},{"id":"family","label":{"en":"Family Bed","es":"Cama Familiar"},"icon":"family","sublabel":{"en":"Kids, pets, or both","es":"Niños, mascotas, o ambos"},"scores":{"durability":2,"motionIsolation":1}}]},{"id":"partner_disturbance","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Does your partner's movement wake you up?","es":"¿El movimiento de tu pareja te despierta?"},"helpText":{"en":"The more movement wakes you, the more it shapes your matches and what we suggest testing.","es":"Cuanto más te despierte el movimiento, más influye en tus opciones y en lo que sugerimos probar."},"type":"single","skipIf":{"question":"partner_sleep","answer":"solo"},"options":[{"id":"yes_often","label":{"en":"Yes, Often","es":"Sí, Seguido"},"icon":"motion","sublabel":{"en":"Every movement wakes me","es":"Cada movimiento me despierta"},"scores":{"motionIsolation":4,"hybrid":3,"memory":2}},{"id":"sometimes","label":{"en":"Sometimes","es":"A Veces"},"icon":"combo","sublabel":{"en":"Bigger movements bother me","es":"Los movimientos grandes me molestan"},"scores":{"motionIsolation":3,"hybrid":2}},{"id":"rarely","label":{"en":"Rarely","es":"Rara Vez"},"icon":"check","sublabel":{"en":"Light sleeper but mostly fine","es":"Sueño ligero pero generalmente bien"},"scores":{"motionIsolation":1}},{"id":"not_applicable","label":{"en":"Doesn't Apply","es":"No Aplica"},"icon":"solo","sublabel":{"en":"I sleep alone","es":"Duermo solo"},"scores":{}}]},{"id":"sleep_position","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"How do you usually sleep?","es":"¿Cómo duermes normalmente?"},"helpText":{"en":"This helps us favor pressure relief, support, or a responsive feel.","es":"Esto nos ayuda a priorizar alivio de presión, soporte o una sensación con más respuesta."},"type":"single","options":[{"id":"side","label":{"en":"Side Sleeper","es":"De Lado"},"icon":"side","sublabel":{"en":"Curled up","es":"Acurrucado"},"scores":{"plush":2,"pressureRelief":2,"soft":1}},{"id":"back","label":{"en":"Back Sleeper","es":"Boca Arriba"},"icon":"back","sublabel":{"en":"Flat on back","es":"Acostado de espalda"},"scores":{"support":2,"medium":2,"zoned":1}},{"id":"stomach","label":{"en":"Stomach Sleeper","es":"Boca Abajo"},"icon":"stomach","sublabel":{"en":"Face down","es":"Boca abajo"},"scores":{"firm":2,"support":1}},{"id":"combo","label":{"en":"Combination","es":"Combinación"},"icon":"combo","sublabel":{"en":"Move around","es":"Me muevo mucho"},"scores":{"medium":2,"responsive":2}},{"id":"no_idea","label":{"en":"Not Sure","es":"No Estoy Seguro"},"icon":"question","sublabel":{"en":"I wake up in weird positions","es":"Me despierto en posiciones raras"},"scores":{"medium":2,"responsive":2}}]},{"id":"body_type","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"What weight range should this mattress support?","es":"¿Qué rango de peso debe soportar este colchón?"},"helpText":{"en":"This helps us account for cushioning, support, and durability.","es":"Esto nos ayuda a considerar la amortiguación, el soporte y la durabilidad."},"type":"single","options":[{"id":"petite","label":{"en":"Under 130 lbs","es":"Menos de 130 lbs"},"icon":"cloud","sublabel":{"en":"Light support","es":"Soporte ligero"},"scores":{"plush":2,"soft":1}},{"id":"average","label":{"en":"130 to 200 lbs","es":"130 a 200 lbs"},"icon":"weight","sublabel":{"en":"Standard support","es":"Soporte estándar"},"scores":{"medium":2}},{"id":"athletic","label":{"en":"200 to 230 lbs","es":"200 a 230 lbs"},"icon":"support","sublabel":{"en":"Medium-firm support","es":"Soporte medio-firme"},"scores":{"support":2,"medium":1,"responsive":1}},{"id":"plus","label":{"en":"Over 230 lbs","es":"Más de 230 lbs"},"icon":"support","sublabel":{"en":"Maximum support","es":"Soporte máximo"},"scores":{"firm":2,"support":3,"hybrid":2,"durability":2}},{"id":"different","label":{"en":"Different weight ranges","es":"Rangos de peso diferentes"},"icon":"partner","sublabel":{"en":"Sleepers fall into different ranges","es":"Los durmientes están en rangos diferentes"},"scores":{"medium":2,"support":1,"motionIsolation":2},"hideIf":{"question":"partner_sleep","answer":"solo"}}],"copyVariants":[{"when":{"question":"partner_sleep","answerIn":["partner","family"]},"question":{"en":"What weight range should we match for the sleeper who needs more support?","es":"¿Para qué rango de peso debemos ajustar, según quien necesite más soporte?"},"helpText":{"en":"If you fall into different ranges, choose “Different weight ranges.”","es":"Si están en rangos diferentes, elige “Rangos de peso diferentes”."}}]},{"id":"temperature","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"How do you sleep temperature-wise?","es":"¿Cómo duermes en cuanto a temperatura?"},"helpText":{"en":"If you sleep hot, we favor cooling features in your matches.","es":"Si duermes con calor, priorizamos materiales refrescantes en tus opciones."},"type":"single","options":[{"id":"hot","label":{"en":"I Sleep Hot","es":"Duermo con Calor"},"icon":"flame","sublabel":{"en":"Night sweats, kick off covers","es":"Sudores nocturnos, quito las cobijas"},"scores":{"cooling":3,"hybrid":2}},{"id":"comfortable","label":{"en":"I'm Comfortable","es":"Estoy Cómodo"},"icon":"smile","sublabel":{"en":"No temperature issues","es":"Sin problemas de temperatura"},"scores":{}},{"id":"cold","label":{"en":"I Sleep Cold","es":"Duermo con Frío"},"icon":"snowflake","sublabel":{"en":"Need blankets to warm up","es":"Necesito cobijas para calentarme"},"scores":{"memory":1,"plush":1}},{"id":"opposite","label":{"en":"We're Opposite","es":"Somos Opuestos"},"icon":"hotcold","sublabel":{"en":"One hot, one cold","es":"Uno con calor, otro con frío"},"scores":{"cooling":2,"hybrid":1},"hideIf":{"question":"partner_sleep","answer":"solo"}}]},{"id":"firmness","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"What firmness level do you prefer?","es":"¿Qué nivel de firmeza prefieres?"},"helpText":{"en":"No wrong answer here, just slide to the feel you prefer.","es":"Desliza a tu comodidad ideal"},"type":"slider","min":1,"max":10,"defaultValue":5,"labels":[{"en":"Soft — Sink right in","es":"Suave — Hundirse"},{"en":"Medium","es":"Medio"},{"en":"Firm — Solid support","es":"Firme — Soporte sólido"}]},{"id":"sleep_issues","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Any issues with your current mattress?","es":"¿Algún problema con tu colchón actual?"},"helpText":{"en":"Tap anything you've noticed. These shape which features we favor and what we suggest testing.","es":"Toca lo que hayas notado. Esto define qué características priorizamos y qué sugerimos probar."},"type":"multiple","options":[{"id":"back_pain","label":{"en":"Back Pain","es":"Dolor de Espalda"},"icon":"spine","sublabel":{"en":"Lower or upper back","es":"Espalda baja o alta"},"scores":{"support":3,"zoned":2,"firm":1}},{"id":"hip_pain","label":{"en":"Hip or Shoulder Pain","es":"Dolor de Cadera u Hombro"},"icon":"pressure","sublabel":{"en":"Pressure points","es":"Puntos de presión"},"scores":{"pressureRelief":3,"plush":2}},{"id":"hot","label":{"en":"Sleeping Too Hot","es":"Mucho Calor al Dormir"},"icon":"flame","sublabel":{"en":"Night sweats, overheating","es":"Sudores nocturnos, sobrecalentamiento"},"scores":{"cooling":3,"hybrid":2}},{"id":"tossing","label":{"en":"Tossing &amp; Turning","es":"Dando Vueltas"},"icon":"combo","sublabel":{"en":"Can't get comfortable","es":"No encuentro comodidad"},"scores":{"comfort":2,"medium":1}},{"id":"stiff","label":{"en":"Waking Up Stiff or Sore","es":"Despertar Rígido o Adolorido"},"icon":"stiff","sublabel":{"en":"Morning aches","es":"Dolores matutinos"},"scores":{"pressureRelief":2,"comfort":2}},{"id":"sagging","label":{"en":"Mattress Sagging","es":"Colchón Hundido"},"icon":"sagging","sublabel":{"en":"Dips or indentations","es":"Hundimientos"},"scores":{"durability":2,"quality":2}},{"id":"too_soft","label":{"en":"Mattress Too Soft","es":"Colchón Muy Suave"},"icon":"couch","sublabel":{"en":"Sinking in too much","es":"Me hundo demasiado"},"scores":{"firm":3,"support":2}},{"id":"none","label":{"en":"No Major Issues","es":"Sin Problemas Grandes"},"icon":"check","sublabel":{"en":"Just time for an upgrade","es":"Solo es hora de un cambio"},"scores":{"comfort":1,"quality":1,"durable":1}}]},{"id":"health_conditions","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Anything else going on that affects your sleep?","es":"¿Algo más que afecte tu sueño?"},"helpText":{"en":"Tap any that apply. Some shape your matches; some change what we suggest trying, like an adjustable base or a mattress protector.","es":"Toca lo que aplique. Algunas influyen en tus opciones; otras cambian lo que sugerimos probar, como una base ajustable o un protector de colchón."},"type":"multiple","options":[{"id":"nerve_pain","label":{"en":"Nerve Pain or Tingling","es":"Dolor Nervioso u Hormigueo"},"icon":"lightning","sublabel":{"en":"Shooting pain, numbness","es":"Dolor punzante, entumecimiento"},"scores":{"support":3,"firm":2,"zoned":2}},{"id":"allergies","label":{"en":"Allergies","es":"Alergias"},"icon":"sneeze","sublabel":{"en":"Dust, sneezing, stuffy","es":"Polvo, estornudos, congestión"},"scores":{"hypoallergenic":3}},{"id":"snoring","label":{"en":"Snoring or Sleep Apnea","es":"Ronquidos o Apnea del Sueño"},"icon":"snore","sublabel":{"en":"You or your partner","es":"Tú o tu pareja"},"scores":{"adjustable":3}},{"id":"reflux","label":{"en":"Acid Reflux / Heartburn","es":"Reflujo Ácido / Acidez"},"icon":"flame","sublabel":{"en":"Burns when lying down","es":"Arde al acostarse"},"scores":{"adjustable":3}},{"id":"extra_support","label":{"en":"Need Extra Support","es":"Necesito Soporte Extra"},"icon":"weight","sublabel":{"en":"Larger build or heavier weight","es":"Complexión grande o peso mayor"},"scores":{"support":3,"firm":2,"durable":3}},{"id":"getting_older","label":{"en":"Changing Needs","es":"Necesidades Cambiantes"},"icon":"aging","sublabel":{"en":"Looking for gentler support","es":"Buscando soporte más suave"},"scores":{"support":2,"comfort":2,"pressureRelief":1}},{"id":"none","label":{"en":"None of These","es":"Ninguno de Estos"},"icon":"check","sublabel":{"en":"I'm good","es":"Estoy bien"},"scores":{}}]}]}}</t>
         </is>
       </c>
     </row>

</xml_diff>